<commit_message>
updated code structure and made changes for optimization and visual
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\globales_Datenschema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{138EE822-71DC-4352-BE44-D281D8426BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46807889-7309-4DA1-9141-9D4EF97F064C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="88">
   <si>
     <t>location</t>
   </si>
@@ -281,6 +281,15 @@
   </si>
   <si>
     <t>AQ</t>
+  </si>
+  <si>
+    <t>Umrechnung notwendig?</t>
+  </si>
+  <si>
+    <t>ja</t>
+  </si>
+  <si>
+    <t>nein</t>
   </si>
 </sst>
 </file>
@@ -296,7 +305,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -327,8 +336,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -466,11 +481,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -494,6 +548,12 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1011,17 +1071,18 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E32"/>
+  <dimension ref="B2:F32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.5703125" customWidth="1"/>
     <col min="3" max="3" width="39.42578125" customWidth="1"/>
     <col min="4" max="4" width="25.7109375" customWidth="1"/>
     <col min="5" max="5" width="27.85546875" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
         <v>29</v>
@@ -1032,8 +1093,11 @@
       <c r="E3" s="10" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F3" s="25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1046,8 +1110,11 @@
       <c r="E4" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
@@ -1060,8 +1127,11 @@
       <c r="E5" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>2</v>
       </c>
@@ -1074,8 +1144,11 @@
       <c r="E6" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
@@ -1088,8 +1161,11 @@
       <c r="E7" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
@@ -1102,8 +1178,11 @@
       <c r="E8" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>5</v>
       </c>
@@ -1116,8 +1195,11 @@
       <c r="E9" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F9" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1130,8 +1212,11 @@
       <c r="E10" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F10" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>7</v>
       </c>
@@ -1144,8 +1229,11 @@
       <c r="E11" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
@@ -1158,8 +1246,11 @@
       <c r="E12" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>9</v>
       </c>
@@ -1172,8 +1263,11 @@
       <c r="E13" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>10</v>
       </c>
@@ -1186,8 +1280,11 @@
       <c r="E14" s="2" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
         <v>11</v>
       </c>
@@ -1200,8 +1297,11 @@
       <c r="E15" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
         <v>12</v>
       </c>
@@ -1214,8 +1314,11 @@
       <c r="E16" s="2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>13</v>
       </c>
@@ -1228,8 +1331,11 @@
       <c r="E17" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>14</v>
       </c>
@@ -1242,8 +1348,11 @@
       <c r="E18" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>15</v>
       </c>
@@ -1256,8 +1365,11 @@
       <c r="E19" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>16</v>
       </c>
@@ -1270,8 +1382,11 @@
       <c r="E20" s="2" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
         <v>17</v>
       </c>
@@ -1284,8 +1399,11 @@
       <c r="E21" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>18</v>
       </c>
@@ -1298,8 +1416,11 @@
       <c r="E22" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>19</v>
       </c>
@@ -1312,8 +1433,11 @@
       <c r="E23" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
         <v>20</v>
       </c>
@@ -1326,8 +1450,11 @@
       <c r="E24" s="2" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
         <v>21</v>
       </c>
@@ -1340,8 +1467,11 @@
       <c r="E25" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F25" s="27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="19" t="s">
         <v>22</v>
       </c>
@@ -1350,8 +1480,9 @@
       </c>
       <c r="D26" s="15"/>
       <c r="E26" s="16"/>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F26" s="23"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
         <v>23</v>
       </c>
@@ -1364,8 +1495,11 @@
       <c r="E27" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>24</v>
       </c>
@@ -1378,8 +1512,11 @@
       <c r="E28" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F28" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
         <v>25</v>
       </c>
@@ -1392,8 +1529,11 @@
       <c r="E29" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F29" s="27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="19" t="s">
         <v>26</v>
       </c>
@@ -1402,8 +1542,9 @@
       </c>
       <c r="D30" s="15"/>
       <c r="E30" s="16"/>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="23"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="19" t="s">
         <v>27</v>
       </c>
@@ -1412,8 +1553,9 @@
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="16"/>
-    </row>
-    <row r="32" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F31" s="23"/>
+    </row>
+    <row r="32" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="20" t="s">
         <v>28</v>
       </c>
@@ -1422,6 +1564,7 @@
       </c>
       <c r="D32" s="17"/>
       <c r="E32" s="18"/>
+      <c r="F32" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added map for first dataset - changes global datascheme to longitude and latitude for global purposes
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\globales_Datenschema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46807889-7309-4DA1-9141-9D4EF97F064C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C29A26-C98E-47B5-A1DE-A03462FA5B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="88">
   <si>
     <t>location</t>
   </si>
@@ -34,12 +34,6 @@
     <t>well_or_spring_name</t>
   </si>
   <si>
-    <t>utm_e</t>
-  </si>
-  <si>
-    <t>utm_n</t>
-  </si>
-  <si>
     <t>depth_bgl_in_m</t>
   </si>
   <si>
@@ -290,6 +284,12 @@
   </si>
   <si>
     <t>nein</t>
+  </si>
+  <si>
+    <t>WGS84_latitude</t>
+  </si>
+  <si>
+    <t>WGS84_longitude</t>
   </si>
 </sst>
 </file>
@@ -550,7 +550,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
@@ -834,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B40B4A1F-305E-4A10-9B22-5AB123015450}">
-  <dimension ref="B2:E32"/>
+  <dimension ref="B2:F32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" customWidth="1"/>
@@ -842,224 +842,257 @@
     <col min="3" max="3" width="31.7109375" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
     <col min="5" max="5" width="28.28515625" customWidth="1"/>
+    <col min="6" max="6" width="27.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F3" s="25" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="6"/>
       <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="23"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="6"/>
       <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="23"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>2</v>
+        <v>86</v>
       </c>
       <c r="C6" s="6"/>
       <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="23"/>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>3</v>
+        <v>87</v>
       </c>
       <c r="C7" s="6"/>
       <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="23"/>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C8" s="6"/>
       <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="23"/>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C9" s="6"/>
       <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F9" s="23"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C10" s="6"/>
       <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F10" s="23"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C11" s="6"/>
       <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="23"/>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C12" s="6"/>
       <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="23"/>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C13" s="6"/>
       <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="23"/>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C14" s="6"/>
       <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="23"/>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C15" s="6"/>
       <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="23"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C16" s="6"/>
       <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="23"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C17" s="6"/>
       <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="23"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C18" s="6"/>
       <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="23"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C19" s="6"/>
       <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="23"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C20" s="6"/>
       <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="23"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C21" s="6"/>
       <c r="E21" s="2"/>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="23"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C22" s="6"/>
       <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="23"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C23" s="6"/>
       <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="23"/>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C24" s="6"/>
       <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="23"/>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C25" s="6"/>
       <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F25" s="23"/>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C26" s="6"/>
       <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F26" s="23"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C27" s="6"/>
       <c r="E27" s="2"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="23"/>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C28" s="6"/>
       <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F28" s="23"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C29" s="6"/>
       <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F29" s="23"/>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C30" s="6"/>
       <c r="E30" s="2"/>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="23"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C31" s="6"/>
       <c r="E31" s="2"/>
-    </row>
-    <row r="32" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F31" s="23"/>
+    </row>
+    <row r="32" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="4"/>
       <c r="E32" s="5"/>
+      <c r="F32" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1085,16 +1118,16 @@
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>31</v>
-      </c>
       <c r="F3" s="25" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
@@ -1102,16 +1135,16 @@
         <v>0</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="F4" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -1119,364 +1152,364 @@
         <v>1</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>2</v>
+        <v>86</v>
       </c>
       <c r="C6" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="26" t="s">
-        <v>86</v>
+      <c r="F6" s="28" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>3</v>
+        <v>87</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="26" t="s">
-        <v>86</v>
+      <c r="F7" s="28" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C10" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D10" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="F10" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F11" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F14" s="28" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D17" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F17" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F18" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F19" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D20" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F20" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D21" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F21" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F22" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D23" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F23" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D24" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F24" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D25" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D26" s="15"/>
       <c r="E26" s="16"/>
@@ -1484,61 +1517,61 @@
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D27" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F27" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D28" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F28" s="26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D29" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F29" s="27" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D30" s="15"/>
       <c r="E30" s="16"/>
@@ -1546,10 +1579,10 @@
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="16"/>
@@ -1557,10 +1590,10 @@
     </row>
     <row r="32" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="20" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D32" s="17"/>
       <c r="E32" s="18"/>

</xml_diff>

<commit_message>
Added yesterdays changes to git
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\globales_Datenschema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C29A26-C98E-47B5-A1DE-A03462FA5B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6CFED53-F39F-468B-90B5-709E5C861814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="2" r:id="rId1"/>
-    <sheet name="REFLECT Datenbank" sheetId="1" r:id="rId2"/>
+    <sheet name="USGS" sheetId="5" r:id="rId2"/>
+    <sheet name="MDPI_Tibet" sheetId="4" r:id="rId3"/>
+    <sheet name="CAES2014" sheetId="3" r:id="rId4"/>
+    <sheet name="REFLECT" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="188">
   <si>
     <t>location</t>
   </si>
@@ -290,6 +293,306 @@
   </si>
   <si>
     <t>WGS84_longitude</t>
+  </si>
+  <si>
+    <t>County</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>SamplingFeatureName</t>
+  </si>
+  <si>
+    <t>LatDegree</t>
+  </si>
+  <si>
+    <t>LongDegree</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>DrilledDepth_ft</t>
+  </si>
+  <si>
+    <t>ja | von ft in m</t>
+  </si>
+  <si>
+    <t>FluidTemperature_C</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>ph_Field</t>
+  </si>
+  <si>
+    <t>AK</t>
+  </si>
+  <si>
+    <t>TotalDissolvedSolids_mgL</t>
+  </si>
+  <si>
+    <t>ja | Addition der mmol/L</t>
+  </si>
+  <si>
+    <t>Na_mgL</t>
+  </si>
+  <si>
+    <t>DC</t>
+  </si>
+  <si>
+    <t>Mg_mgL</t>
+  </si>
+  <si>
+    <t>DB</t>
+  </si>
+  <si>
+    <t>ja | in mmol/L</t>
+  </si>
+  <si>
+    <t>Ca_mgL</t>
+  </si>
+  <si>
+    <t>CX</t>
+  </si>
+  <si>
+    <t>Cl_mgL</t>
+  </si>
+  <si>
+    <t>CY</t>
+  </si>
+  <si>
+    <t>SO4_mgL</t>
+  </si>
+  <si>
+    <t>DF</t>
+  </si>
+  <si>
+    <t>K_mgL</t>
+  </si>
+  <si>
+    <t>DA</t>
+  </si>
+  <si>
+    <t>Sr_mgL</t>
+  </si>
+  <si>
+    <t>EB</t>
+  </si>
+  <si>
+    <t>ja | in μmol/L</t>
+  </si>
+  <si>
+    <t>F_mgL</t>
+  </si>
+  <si>
+    <t>CZ</t>
+  </si>
+  <si>
+    <t>Li_mgL</t>
+  </si>
+  <si>
+    <t>CH</t>
+  </si>
+  <si>
+    <t>Alkalinity_mgL</t>
+  </si>
+  <si>
+    <t>DI</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>nicht vorhanden - IDAHO eintragen</t>
+  </si>
+  <si>
+    <t>Longitude</t>
+  </si>
+  <si>
+    <t>Latitude</t>
+  </si>
+  <si>
+    <t>Sheet1</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Temperature_C</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>Conductivity_uS_cm</t>
+  </si>
+  <si>
+    <t>nicht vorhanden, wird berechnet</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>ja | Addition in mmol/L</t>
+  </si>
+  <si>
+    <t>HCO3_mgL</t>
+  </si>
+  <si>
+    <t>Li_ugL</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>Sr_ugL</t>
+  </si>
+  <si>
+    <t>Fe_ugL</t>
+  </si>
+  <si>
+    <t>AD</t>
+  </si>
+  <si>
+    <t>Mn_ugL</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>NO3_mgL</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>COUNTY</t>
+  </si>
+  <si>
+    <t>WELLNAME</t>
+  </si>
+  <si>
+    <t>LATITUDE</t>
+  </si>
+  <si>
+    <t>LONGITUDE</t>
+  </si>
+  <si>
+    <t>PERIOD</t>
+  </si>
+  <si>
+    <t>DEPTHLOWER</t>
+  </si>
+  <si>
+    <t>PH</t>
+  </si>
+  <si>
+    <t>TEMP</t>
+  </si>
+  <si>
+    <t>nein, wenige Daten</t>
+  </si>
+  <si>
+    <t>LITHOLOGY</t>
+  </si>
+  <si>
+    <t>TDS</t>
+  </si>
+  <si>
+    <t>ja | Addition der mmol/L  | ACHTUNG - ähnliches Attribut TSUSGS</t>
+  </si>
+  <si>
+    <t>HCO3</t>
+  </si>
+  <si>
+    <t>CE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ja | in mmol/L  </t>
+  </si>
+  <si>
+    <t>Cl</t>
+  </si>
+  <si>
+    <t>SO4</t>
+  </si>
+  <si>
+    <t>Li</t>
+  </si>
+  <si>
+    <t>Sr</t>
+  </si>
+  <si>
+    <t>Mn</t>
+  </si>
+  <si>
+    <t>NO3</t>
+  </si>
+  <si>
+    <t>HS</t>
+  </si>
+  <si>
+    <t>Ca</t>
+  </si>
+  <si>
+    <t>CF</t>
+  </si>
+  <si>
+    <t>CM</t>
+  </si>
+  <si>
+    <t>FeTot</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>CV</t>
+  </si>
+  <si>
+    <t>Mg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ja | in μmol/L  </t>
+  </si>
+  <si>
+    <t>DY</t>
+  </si>
+  <si>
+    <t>DD</t>
+  </si>
+  <si>
+    <t>DS</t>
+  </si>
+  <si>
+    <t>DR</t>
+  </si>
+  <si>
+    <t>Na</t>
+  </si>
+  <si>
+    <t>DH</t>
   </si>
 </sst>
 </file>
@@ -305,7 +608,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -342,8 +645,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -520,11 +829,224 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -554,6 +1076,41 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -958,60 +1515,57 @@
       <c r="F15" s="23"/>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="39" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="6"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="23"/>
+      <c r="F16" s="41"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="23"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="40"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="39" t="s">
         <v>12</v>
       </c>
       <c r="C18" s="6"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="23"/>
+      <c r="F18" s="41"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="39" t="s">
         <v>13</v>
       </c>
       <c r="C19" s="6"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="23"/>
+      <c r="F19" s="41"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="39" t="s">
         <v>14</v>
       </c>
       <c r="C20" s="6"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="23"/>
+      <c r="F20" s="41"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="39" t="s">
         <v>15</v>
       </c>
       <c r="C21" s="6"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="23"/>
+      <c r="F21" s="41"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="23"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="46"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
@@ -1100,6 +1654,1450 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85E326E-8D3B-4CF5-91CA-01DA393CBB40}">
+  <dimension ref="B2:I32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="36.85546875" customWidth="1"/>
+    <col min="3" max="3" width="31.7109375" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
+    <col min="5" max="5" width="28.7109375" customWidth="1"/>
+    <col min="6" max="6" width="59.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="11"/>
+      <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="D4" t="s">
+        <v>134</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" t="s">
+        <v>134</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="D6" t="s">
+        <v>134</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="D7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F7" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D10" t="s">
+        <v>134</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="15"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="29"/>
+      <c r="I12" s="61"/>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="D13" t="s">
+        <v>134</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="15"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="29"/>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D15" t="s">
+        <v>134</v>
+      </c>
+      <c r="E15" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" s="26" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="48"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>186</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>187</v>
+      </c>
+      <c r="F17" s="63" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D18" t="s">
+        <v>134</v>
+      </c>
+      <c r="E18" t="s">
+        <v>116</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D19" t="s">
+        <v>134</v>
+      </c>
+      <c r="E19" t="s">
+        <v>175</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D20" t="s">
+        <v>134</v>
+      </c>
+      <c r="E20" t="s">
+        <v>127</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D21" t="s">
+        <v>134</v>
+      </c>
+      <c r="E21" t="s">
+        <v>185</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>164</v>
+      </c>
+      <c r="D22" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>165</v>
+      </c>
+      <c r="F22" s="43" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D23" s="59" t="s">
+        <v>134</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F23" s="60" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D25" t="s">
+        <v>134</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F25" s="26" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="6"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="26" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D27" t="s">
+        <v>134</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D28" t="s">
+        <v>171</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D29" t="s">
+        <v>134</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="F29" s="26" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="D30" t="s">
+        <v>134</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="F30" s="26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="29"/>
+    </row>
+    <row r="32" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="F32" s="62" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC28484C-C581-4663-8490-31B7BD27263E}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:F32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="36.7109375" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" customWidth="1"/>
+    <col min="5" max="5" width="28.7109375" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="11"/>
+      <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4" t="s">
+        <v>134</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D5" t="s">
+        <v>134</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D6" t="s">
+        <v>134</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F7" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="15"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="29"/>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="15"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="29"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="15"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="29"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12" t="s">
+        <v>134</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>134</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="15"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="26" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="49" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="50" t="s">
+        <v>139</v>
+      </c>
+      <c r="D15" s="51"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="53"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="48"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>140</v>
+      </c>
+      <c r="F17" s="45" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" t="s">
+        <v>134</v>
+      </c>
+      <c r="E18" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" t="s">
+        <v>134</v>
+      </c>
+      <c r="E19" t="s">
+        <v>80</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" t="s">
+        <v>134</v>
+      </c>
+      <c r="E20" t="s">
+        <v>77</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="D21" t="s">
+        <v>134</v>
+      </c>
+      <c r="E21" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>142</v>
+      </c>
+      <c r="D22" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="F22" s="43" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D23" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" s="45" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D25" t="s">
+        <v>134</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F25" s="26" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="15"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="29"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="D27" t="s">
+        <v>134</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D28" t="s">
+        <v>134</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D29" t="s">
+        <v>134</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F29" s="26" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D30" t="s">
+        <v>134</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F30" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="29" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="55" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="56"/>
+      <c r="E32" s="57"/>
+      <c r="F32" s="58" t="s">
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="79" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{783802C3-70F2-469E-9F15-66886A2B472E}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:F32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="40.140625" customWidth="1"/>
+    <col min="3" max="3" width="30.42578125" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="5" max="5" width="28.5703125" customWidth="1"/>
+    <col min="6" max="6" width="29.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="11"/>
+      <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" t="s">
+        <v>90</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F8" s="26" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="15"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="29"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="15"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="29"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" t="s">
+        <v>90</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="16"/>
+      <c r="F12" s="29"/>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="15"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="29"/>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="26" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="15"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="29"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="F17" s="45" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="D21" t="s">
+        <v>90</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>128</v>
+      </c>
+      <c r="D22" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="F22" s="43" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D23" t="s">
+        <v>90</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F23" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D24" t="s">
+        <v>90</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D25" t="s">
+        <v>90</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F25" s="26" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="15"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="29"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27" s="15"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="29"/>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D28" s="15"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="29"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D29" t="s">
+        <v>90</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F29" s="26" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" s="15"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="29"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B31" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="29"/>
+    </row>
+    <row r="32" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="17"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="31"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="79" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -1352,19 +3350,19 @@
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="F17" s="26" t="s">
+      <c r="F17" s="45" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1437,19 +3435,19 @@
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="F22" s="26" t="s">
+      <c r="F22" s="43" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added second database - American USGS Databse with 135.000 data points
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\globales_Datenschema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6CFED53-F39F-468B-90B5-709E5C861814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09838B02-C711-4762-BB9F-A9CD21780430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="2" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="CAES2014" sheetId="3" r:id="rId4"/>
     <sheet name="REFLECT" sheetId="1" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="189">
   <si>
     <t>location</t>
   </si>
@@ -593,6 +593,9 @@
   </si>
   <si>
     <t>DH</t>
+  </si>
+  <si>
+    <t>NH4</t>
   </si>
 </sst>
 </file>
@@ -1046,7 +1049,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1106,9 +1109,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
@@ -1655,7 +1655,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85E326E-8D3B-4CF5-91CA-01DA393CBB40}">
-  <dimension ref="B2:I32"/>
+  <dimension ref="B2:F32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" customWidth="1"/>
@@ -1665,8 +1665,8 @@
     <col min="6" max="6" width="59.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
         <v>27</v>
@@ -1681,7 +1681,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
@@ -1715,7 +1715,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>86</v>
       </c>
@@ -1732,7 +1732,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>87</v>
       </c>
@@ -1749,7 +1749,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>3</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>4</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="19" t="s">
         <v>6</v>
       </c>
@@ -1827,9 +1827,8 @@
       <c r="D12" s="15"/>
       <c r="E12" s="16"/>
       <c r="F12" s="29"/>
-      <c r="I12" s="61"/>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>7</v>
       </c>
@@ -1846,7 +1845,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="19" t="s">
         <v>8</v>
       </c>
@@ -1857,7 +1856,7 @@
       <c r="E14" s="16"/>
       <c r="F14" s="29"/>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="12" t="s">
         <v>9</v>
       </c>
@@ -1874,7 +1873,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="47" t="s">
         <v>10</v>
       </c>
@@ -1898,7 +1897,7 @@
       <c r="E17" s="33" t="s">
         <v>187</v>
       </c>
-      <c r="F17" s="63" t="s">
+      <c r="F17" s="60" t="s">
         <v>166</v>
       </c>
     </row>
@@ -1994,13 +1993,13 @@
       <c r="C23" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="D23" s="59" t="s">
+      <c r="D23" t="s">
         <v>134</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F23" s="60" t="s">
+      <c r="F23" s="26" t="s">
         <v>166</v>
       </c>
     </row>
@@ -2042,8 +2041,15 @@
       <c r="B26" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="E26" s="2"/>
+      <c r="C26" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D26" t="s">
+        <v>134</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>118</v>
+      </c>
       <c r="F26" s="26" t="s">
         <v>181</v>
       </c>
@@ -2140,7 +2146,7 @@
       <c r="E32" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="F32" s="62" t="s">
+      <c r="F32" s="59" t="s">
         <v>166</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added another database and implemented combination of databases
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\globales_Datenschema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50595504-BEC3-4E0D-BFEC-5F6ACF63229A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3745E880-0F6C-46B5-829B-3D2A81E2C200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="2" r:id="rId1"/>
-    <sheet name="USGS" sheetId="5" r:id="rId2"/>
-    <sheet name="MDPI_Tibet" sheetId="4" r:id="rId3"/>
-    <sheet name="CAES2014" sheetId="3" r:id="rId4"/>
-    <sheet name="REFLECT" sheetId="1" r:id="rId5"/>
+    <sheet name="ALPS" sheetId="6" r:id="rId2"/>
+    <sheet name="USGS" sheetId="5" r:id="rId3"/>
+    <sheet name="MDPI_Tibet" sheetId="4" r:id="rId4"/>
+    <sheet name="CAES2014" sheetId="3" r:id="rId5"/>
+    <sheet name="REFLECT" sheetId="1" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="162913" concurrentCalc="0"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="218">
   <si>
     <t>location</t>
   </si>
@@ -605,6 +606,84 @@
   </si>
   <si>
     <t>manche Daten in ppm, ausgehen von mg/L = ppm, da Dichte unbekannt</t>
+  </si>
+  <si>
+    <t>CAES2014</t>
+  </si>
+  <si>
+    <t>REFLECT</t>
+  </si>
+  <si>
+    <t>MDPI Tibet</t>
+  </si>
+  <si>
+    <t>USGS</t>
+  </si>
+  <si>
+    <t>ALPS</t>
+  </si>
+  <si>
+    <t>spring location</t>
+  </si>
+  <si>
+    <t>spring name</t>
+  </si>
+  <si>
+    <t>longitude</t>
+  </si>
+  <si>
+    <t>latitude</t>
+  </si>
+  <si>
+    <t>well_depth_(m)</t>
+  </si>
+  <si>
+    <t>Na_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>Ca_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>Mg_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>Cl_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>HCO3_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>SO4_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>Li_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>temperature_(degr_C)</t>
+  </si>
+  <si>
+    <t>EC_(S_m^-1)</t>
+  </si>
+  <si>
+    <t>TDS_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>K_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>NH4_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>F_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>NO3_(mg L^-1)</t>
+  </si>
+  <si>
+    <t>lithology</t>
+  </si>
+  <si>
+    <t>ja | von S/m in uS/cm</t>
   </si>
 </sst>
 </file>
@@ -670,7 +749,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -1060,11 +1139,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1126,10 +1216,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1616,7 +1705,7 @@
       <c r="C23" s="6"/>
       <c r="E23" s="2"/>
       <c r="F23" s="23"/>
-      <c r="G23" s="62"/>
+      <c r="G23" s="23"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
@@ -1625,7 +1714,7 @@
       <c r="C24" s="6"/>
       <c r="E24" s="2"/>
       <c r="F24" s="23"/>
-      <c r="G24" s="63"/>
+      <c r="G24" s="23"/>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
@@ -1634,7 +1723,7 @@
       <c r="C25" s="6"/>
       <c r="E25" s="2"/>
       <c r="F25" s="23"/>
-      <c r="G25" s="62"/>
+      <c r="G25" s="23"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
@@ -1643,7 +1732,7 @@
       <c r="C26" s="6"/>
       <c r="E26" s="2"/>
       <c r="F26" s="23"/>
-      <c r="G26" s="63"/>
+      <c r="G26" s="23"/>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
@@ -1652,7 +1741,7 @@
       <c r="C27" s="6"/>
       <c r="E27" s="2"/>
       <c r="F27" s="23"/>
-      <c r="G27" s="62"/>
+      <c r="G27" s="23"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
@@ -1661,7 +1750,7 @@
       <c r="C28" s="6"/>
       <c r="E28" s="2"/>
       <c r="F28" s="23"/>
-      <c r="G28" s="62"/>
+      <c r="G28" s="23"/>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
@@ -1706,6 +1795,416 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2F6DB8F-FD5C-4693-8887-04E42CDC7E06}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:G32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="3" max="3" width="29.85546875" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="23"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G5" s="23"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G6" s="23"/>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G7" s="23"/>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G8" s="23"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G9" s="23"/>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="15"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G11" s="23"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="26" t="s">
+        <v>217</v>
+      </c>
+      <c r="G12" s="23"/>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="23"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" s="15"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" s="23"/>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="29"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>202</v>
+      </c>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G17" s="23"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G18" s="23"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G19" s="23"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G20" s="23"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G21" s="23"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>206</v>
+      </c>
+      <c r="D22" s="36"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G22" s="23"/>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="E23" s="2"/>
+      <c r="F23" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G23" s="23"/>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G24" s="23"/>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D25" s="15"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="29"/>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="G26" s="23"/>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27" s="15"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D28" s="15"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="E29" s="2"/>
+      <c r="F29" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="G29" s="23"/>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="E30" s="2"/>
+      <c r="F30" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="G30" s="23"/>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="15"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+    </row>
+    <row r="32" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="63" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32" s="17"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="31"/>
+      <c r="G32" s="31"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="70" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85E326E-8D3B-4CF5-91CA-01DA393CBB40}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -1723,7 +2222,9 @@
   <sheetData>
     <row r="2" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="11"/>
+      <c r="B3" s="11" t="s">
+        <v>195</v>
+      </c>
       <c r="C3" s="8" t="s">
         <v>27</v>
       </c>
@@ -2266,7 +2767,7 @@
       <c r="F32" s="59" t="s">
         <v>166</v>
       </c>
-      <c r="G32" s="64" t="s">
+      <c r="G32" s="62" t="s">
         <v>191</v>
       </c>
     </row>
@@ -2276,7 +2777,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC28484C-C581-4663-8490-31B7BD27263E}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -2294,7 +2795,9 @@
   <sheetData>
     <row r="2" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="11"/>
+      <c r="B3" s="11" t="s">
+        <v>194</v>
+      </c>
       <c r="C3" s="8" t="s">
         <v>27</v>
       </c>
@@ -2799,7 +3302,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{783802C3-70F2-469E-9F15-66886A2B472E}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -2816,7 +3319,9 @@
   <sheetData>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="11"/>
+      <c r="B3" s="11" t="s">
+        <v>192</v>
+      </c>
       <c r="C3" s="8" t="s">
         <v>27</v>
       </c>
@@ -3265,7 +3770,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3282,7 +3787,9 @@
   <sheetData>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="11"/>
+      <c r="B3" s="11" t="s">
+        <v>193</v>
+      </c>
       <c r="C3" s="8" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Tried adding more databases
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
@@ -8,29 +8,40 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\globales_Datenschema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3745E880-0F6C-46B5-829B-3D2A81E2C200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1697FD-B7AB-42A5-A17E-92AFC57BFC97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="2" r:id="rId1"/>
-    <sheet name="ALPS" sheetId="6" r:id="rId2"/>
-    <sheet name="USGS" sheetId="5" r:id="rId3"/>
-    <sheet name="MDPI_Tibet" sheetId="4" r:id="rId4"/>
-    <sheet name="CAES2014" sheetId="3" r:id="rId5"/>
-    <sheet name="REFLECT" sheetId="1" r:id="rId6"/>
+    <sheet name="HESSEN" sheetId="7" r:id="rId2"/>
+    <sheet name="MOESM2" sheetId="8" r:id="rId3"/>
+    <sheet name="ALPS" sheetId="6" r:id="rId4"/>
+    <sheet name="USGS" sheetId="5" r:id="rId5"/>
+    <sheet name="MDPI_Tibet" sheetId="4" r:id="rId6"/>
+    <sheet name="CAES2014" sheetId="3" r:id="rId7"/>
+    <sheet name="REFLECT" sheetId="1" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="271">
   <si>
     <t>location</t>
   </si>
@@ -684,6 +695,165 @@
   </si>
   <si>
     <t>ja | von S/m in uS/cm</t>
+  </si>
+  <si>
+    <t>ja | ist in Zahlen kodiert</t>
+  </si>
+  <si>
+    <t>Town</t>
+  </si>
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>Well or Spring Name</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Zeile 3</t>
+  </si>
+  <si>
+    <t>ja | in Long und Lat</t>
+  </si>
+  <si>
+    <t>Coordinates R</t>
+  </si>
+  <si>
+    <t>Coordinates H</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>Final depth</t>
+  </si>
+  <si>
+    <t>Rock type</t>
+  </si>
+  <si>
+    <t>Zeile 4</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>Electric</t>
+  </si>
+  <si>
+    <t>Temperature</t>
+  </si>
+  <si>
+    <t>AF</t>
+  </si>
+  <si>
+    <t>Zeile 3 + 5 Kombi</t>
+  </si>
+  <si>
+    <t>AH</t>
+  </si>
+  <si>
+    <t>Redox</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>Total dissolved solids calculated</t>
+  </si>
+  <si>
+    <t>As</t>
+  </si>
+  <si>
+    <t>Egal, wird später berechnet</t>
+  </si>
+  <si>
+    <t>Sodium</t>
+  </si>
+  <si>
+    <t>AU</t>
+  </si>
+  <si>
+    <t>Magnesium</t>
+  </si>
+  <si>
+    <t>Calcium</t>
+  </si>
+  <si>
+    <t>Chloride</t>
+  </si>
+  <si>
+    <t>Sulphate</t>
+  </si>
+  <si>
+    <t>Bicarbonate</t>
+  </si>
+  <si>
+    <t>AZ</t>
+  </si>
+  <si>
+    <t>Lithium</t>
+  </si>
+  <si>
+    <t>Potassium</t>
+  </si>
+  <si>
+    <t>Strontium</t>
+  </si>
+  <si>
+    <t>Ammonium</t>
+  </si>
+  <si>
+    <t>Iron</t>
+  </si>
+  <si>
+    <t>Manganese</t>
+  </si>
+  <si>
+    <t>Fluoride</t>
+  </si>
+  <si>
+    <t>Nitrate</t>
+  </si>
+  <si>
+    <t>Silica</t>
+  </si>
+  <si>
+    <t>Oxigen</t>
+  </si>
+  <si>
+    <t>BB</t>
+  </si>
+  <si>
+    <t>BD</t>
+  </si>
+  <si>
+    <t>BG</t>
+  </si>
+  <si>
+    <t>BJ</t>
+  </si>
+  <si>
+    <t>BM</t>
+  </si>
+  <si>
+    <t>???????????</t>
+  </si>
+  <si>
+    <t>?????????????</t>
+  </si>
+  <si>
+    <t>Table1</t>
+  </si>
+  <si>
+    <t>MOESM2 (vsl. nicht nutzbar)</t>
+  </si>
+  <si>
+    <t>Hessen (muss angepasst werden)</t>
+  </si>
+  <si>
+    <t>zu wenig Daten</t>
   </si>
 </sst>
 </file>
@@ -1154,7 +1324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1219,6 +1389,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1795,6 +1966,966 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A059286-C8A1-4672-9077-497707963BB5}">
+  <dimension ref="B2:G32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="36.28515625" customWidth="1"/>
+    <col min="3" max="3" width="31.140625" customWidth="1"/>
+    <col min="4" max="4" width="27" customWidth="1"/>
+    <col min="5" max="5" width="29.5703125" customWidth="1"/>
+    <col min="6" max="6" width="25.28515625" customWidth="1"/>
+    <col min="7" max="7" width="27" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D4" t="s">
+        <v>220</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="D5" t="s">
+        <v>220</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G5" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D6" t="s">
+        <v>220</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="F6" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="D7" t="s">
+        <v>220</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="G7" s="23" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D8" t="s">
+        <v>220</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="D9" t="s">
+        <v>220</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F9" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D10" t="s">
+        <v>220</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F10" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="23" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="D11" t="s">
+        <v>220</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G11" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="D12" t="s">
+        <v>220</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G12" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>220</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="D14" t="s">
+        <v>220</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D15" t="s">
+        <v>220</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="F15" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="D16" t="s">
+        <v>220</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="F16" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>242</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>220</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>243</v>
+      </c>
+      <c r="F17" s="60" t="s">
+        <v>166</v>
+      </c>
+      <c r="G17" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="D18" t="s">
+        <v>220</v>
+      </c>
+      <c r="E18" t="s">
+        <v>52</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="D19" t="s">
+        <v>220</v>
+      </c>
+      <c r="E19" t="s">
+        <v>54</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="D20" t="s">
+        <v>220</v>
+      </c>
+      <c r="E20" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G20" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="D21" t="s">
+        <v>220</v>
+      </c>
+      <c r="E21" t="s">
+        <v>58</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G21" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>248</v>
+      </c>
+      <c r="D22" s="36" t="s">
+        <v>220</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>249</v>
+      </c>
+      <c r="F22" s="43" t="s">
+        <v>166</v>
+      </c>
+      <c r="G22" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="D23" s="33" t="s">
+        <v>220</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G23" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="D24" t="s">
+        <v>220</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G24" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D25" t="s">
+        <v>220</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F25" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="G25" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="D26" t="s">
+        <v>220</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="F26" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="D27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G27" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="D28" t="s">
+        <v>220</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G28" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="D29" t="s">
+        <v>220</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="G29" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="D30" t="s">
+        <v>220</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="F30" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G30" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="D31" t="s">
+        <v>220</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="F31" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="G31" s="23" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F32" s="59" t="s">
+        <v>166</v>
+      </c>
+      <c r="G32" s="24" t="s">
+        <v>223</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF8011DF-EFF6-4FCD-84E2-B9EE254EAD4E}">
+  <dimension ref="B2:G32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="37.28515625" customWidth="1"/>
+    <col min="3" max="3" width="32.140625" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="30.28515625" customWidth="1"/>
+    <col min="7" max="7" width="32.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D4" t="s">
+        <v>267</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="23"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="6"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="6"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="6"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="6"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="6"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="6"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="6"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="32"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="6"/>
+      <c r="F18" s="41"/>
+      <c r="G18" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="6"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="6"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="35"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="6"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="6"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="6"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="6"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="6"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="6"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="6"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="7"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24" t="s">
+        <v>270</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2F6DB8F-FD5C-4693-8887-04E42CDC7E06}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -1904,8 +3035,8 @@
         <v>216</v>
       </c>
       <c r="E9" s="2"/>
-      <c r="F9" s="28" t="s">
-        <v>85</v>
+      <c r="F9" s="26" t="s">
+        <v>218</v>
       </c>
       <c r="G9" s="23"/>
     </row>
@@ -2204,7 +3335,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85E326E-8D3B-4CF5-91CA-01DA393CBB40}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -2777,7 +3908,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC28484C-C581-4663-8490-31B7BD27263E}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3302,7 +4433,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{783802C3-70F2-469E-9F15-66886A2B472E}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3770,7 +4901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>

</xml_diff>

<commit_message>
Added more Databases to Collection of Datasets
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\globales_Datenschema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1697FD-B7AB-42A5-A17E-92AFC57BFC97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE9EF0BC-B2FB-4984-BFFE-776774711319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="2" r:id="rId1"/>
-    <sheet name="HESSEN" sheetId="7" r:id="rId2"/>
-    <sheet name="MOESM2" sheetId="8" r:id="rId3"/>
-    <sheet name="ALPS" sheetId="6" r:id="rId4"/>
-    <sheet name="USGS" sheetId="5" r:id="rId5"/>
-    <sheet name="MDPI_Tibet" sheetId="4" r:id="rId6"/>
-    <sheet name="CAES2014" sheetId="3" r:id="rId7"/>
-    <sheet name="REFLECT" sheetId="1" r:id="rId8"/>
+    <sheet name="|---&gt; nutzbare" sheetId="11" r:id="rId2"/>
+    <sheet name="SVZ_Chile" sheetId="9" r:id="rId3"/>
+    <sheet name="HESSEN" sheetId="7" r:id="rId4"/>
+    <sheet name="ALPS" sheetId="6" r:id="rId5"/>
+    <sheet name="USGS" sheetId="5" r:id="rId6"/>
+    <sheet name="MDPI_Tibet" sheetId="4" r:id="rId7"/>
+    <sheet name="CAES2014" sheetId="3" r:id="rId8"/>
+    <sheet name="REFLECT" sheetId="1" r:id="rId9"/>
+    <sheet name="|---&gt; nicht nutzbare" sheetId="10" r:id="rId10"/>
+    <sheet name="MOESM2" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="290">
   <si>
     <t>location</t>
   </si>
@@ -854,6 +857,63 @@
   </si>
   <si>
     <t>zu wenig Daten</t>
+  </si>
+  <si>
+    <t>Location_name</t>
+  </si>
+  <si>
+    <t>Table1_Merged</t>
+  </si>
+  <si>
+    <t>Fault_domain</t>
+  </si>
+  <si>
+    <t>Ableiten aus Location_name (grob)</t>
+  </si>
+  <si>
+    <t>t_C</t>
+  </si>
+  <si>
+    <t>TDS_ppm</t>
+  </si>
+  <si>
+    <t>Cl_ppm</t>
+  </si>
+  <si>
+    <t>SO4_ppm</t>
+  </si>
+  <si>
+    <t>HCO3_ppm</t>
+  </si>
+  <si>
+    <t>K_ppm</t>
+  </si>
+  <si>
+    <t>Na_ppm</t>
+  </si>
+  <si>
+    <t>Mg_ppm</t>
+  </si>
+  <si>
+    <t>Ca_ppm</t>
+  </si>
+  <si>
+    <t>Li_ppb</t>
+  </si>
+  <si>
+    <t>Sr_ppb</t>
+  </si>
+  <si>
+    <t>Schätzen aus Location_name (grob)</t>
+  </si>
+  <si>
+    <t>liegt in ppb vor, müsste in ppm vorliegen</t>
+  </si>
+  <si>
+    <t>SVZ_Chile</t>
+  </si>
+  <si>
+    <t>W</t>
   </si>
 </sst>
 </file>
@@ -1324,7 +1384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1390,6 +1450,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1965,7 +2026,819 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAAC61E6-50DF-405D-A52F-EDADE72AA266}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF8011DF-EFF6-4FCD-84E2-B9EE254EAD4E}">
+  <dimension ref="B2:G32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="37.28515625" customWidth="1"/>
+    <col min="3" max="3" width="32.140625" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="30.28515625" customWidth="1"/>
+    <col min="7" max="7" width="32.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D4" t="s">
+        <v>267</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="23"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="6"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="6"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="6"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="6"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="6"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="6"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="6"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="32"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="6"/>
+      <c r="F18" s="41"/>
+      <c r="G18" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="6"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="6"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="35"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="6"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="6"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="6"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="6"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="6"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="6"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="6"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="7"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24" t="s">
+        <v>270</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFF34DBC-9B7A-4964-BEA9-A6721237D408}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D46C7FC-4F92-409B-95F3-5697C13BE790}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:G32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="36.140625" customWidth="1"/>
+    <col min="3" max="3" width="30.85546875" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" customWidth="1"/>
+    <col min="7" max="7" width="41.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="D4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="23"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="D5" t="s">
+        <v>272</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G5" s="23"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" s="13"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="13"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="29" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="13"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="13"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="13"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="D11" t="s">
+        <v>272</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G11" s="23"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="13"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>272</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="23"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="D15" t="s">
+        <v>272</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F15" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15" s="23"/>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="13"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>281</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>272</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G17" s="23"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="D18" t="s">
+        <v>272</v>
+      </c>
+      <c r="E18" s="65" t="s">
+        <v>102</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G18" s="23"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="D19" t="s">
+        <v>272</v>
+      </c>
+      <c r="E19" s="65" t="s">
+        <v>77</v>
+      </c>
+      <c r="F19" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G19" s="23"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="D20" t="s">
+        <v>272</v>
+      </c>
+      <c r="E20" s="65" t="s">
+        <v>140</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G20" s="23"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D21" t="s">
+        <v>272</v>
+      </c>
+      <c r="E21" s="65" t="s">
+        <v>144</v>
+      </c>
+      <c r="F21" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G21" s="23"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>279</v>
+      </c>
+      <c r="D22" s="36" t="s">
+        <v>272</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="F22" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G22" s="23"/>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="D23" t="s">
+        <v>272</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F23" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="G23" s="23" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="D24" t="s">
+        <v>272</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F24" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G24" s="23"/>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="D25" t="s">
+        <v>272</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="F25" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="G25" s="23"/>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="13"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="13"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="29"/>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="13"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+    </row>
+    <row r="32" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="14"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="31"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="66" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A059286-C8A1-4672-9077-497707963BB5}">
   <dimension ref="B2:G32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2584,348 +3457,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF8011DF-EFF6-4FCD-84E2-B9EE254EAD4E}">
-  <dimension ref="B2:G32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="37.28515625" customWidth="1"/>
-    <col min="3" max="3" width="32.140625" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="30.28515625" customWidth="1"/>
-    <col min="7" max="7" width="32.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="11" t="s">
-        <v>268</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="G3" s="25" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="D4" t="s">
-        <v>267</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="G4" s="23"/>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="6"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" s="6"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" s="6"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C8" s="6"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="6"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="6"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="6"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="6"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="6"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" s="6"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B15" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="6"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B16" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="38" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="32"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="39" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="6"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B19" s="39" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="6"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="39" t="s">
-        <v>14</v>
-      </c>
-      <c r="C20" s="6"/>
-      <c r="F20" s="41"/>
-      <c r="G20" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="6"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B22" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="C22" s="35"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B23" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" s="6"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B24" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" s="6"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="23"/>
-      <c r="G24" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B25" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C25" s="6"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B26" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C26" s="6"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B27" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C27" s="6"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B28" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C28" s="6"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B29" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C29" s="6"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C30" s="6"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B31" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C31" s="6"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="32" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C32" s="7"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24" t="s">
-        <v>270</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2F6DB8F-FD5C-4693-8887-04E42CDC7E06}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3335,7 +3867,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A85E326E-8D3B-4CF5-91CA-01DA393CBB40}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -3908,7 +4440,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC28484C-C581-4663-8490-31B7BD27263E}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -4433,7 +4965,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{783802C3-70F2-469E-9F15-66886A2B472E}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -4901,7 +5433,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>

</xml_diff>

<commit_message>
Added Hessen and GANDAKI Database
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/globales_Datenschema/Anpassung auf globales Datenschema.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\globales_Datenschema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{797A48E8-599E-4C5B-BACF-4D8EEE0BE0EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC44011C-9519-40EA-9257-19D22C58596B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="960" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="960" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="2" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1670" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1673" uniqueCount="411">
   <si>
     <t>location</t>
   </si>
@@ -1413,7 +1413,7 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Coordinates H -&gt; </t>
+      <t xml:space="preserve">K (mg/L) -&gt; </t>
     </r>
     <r>
       <rPr>
@@ -1424,7 +1424,288 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Coordinates_H</t>
+      <t>K_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Fe (mg/L) -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fe_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Mn (mg/L) -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mn_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Na (mg/L) -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Na_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Mg (mg/L) -&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Mg_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ca (mg/L) -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ca_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cl (mg/L) -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cl_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SO4 (mg/L) -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SO4_mg-l</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">HCO3 (mg/L) -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>HCO3_mg-l</t>
+    </r>
+  </si>
+  <si>
+    <t>Geothermal province -&gt; Geothermal_province</t>
+  </si>
+  <si>
+    <t>Nein, da HCO3 einwertig ist gilt meq/L = mmol/L</t>
+  </si>
+  <si>
+    <r>
+      <t>CLA flow path -&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> CLA_flow_path</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bore/Spring -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bore_Spring</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Mg (mg/L) -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mg_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Ca (mg/L) -&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Ca_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>SO4 (mg/L) -&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> SO4_mg-L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Alkalinity (meq/L) -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Alkalinity_meq-L</t>
+    </r>
+  </si>
+  <si>
+    <t>liegt in ppb vor, müsste in ppm vorliegen, Faktor / 1.000</t>
+  </si>
+  <si>
+    <r>
+      <t>Well or Spring Name -&gt; Well_or_</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Spring_Name</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Final depth -&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Final_depth</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Rock type -&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Rock_type</t>
     </r>
   </si>
   <si>
@@ -1442,10 +1723,20 @@
       </rPr>
       <t>Coordinates_R</t>
     </r>
-  </si>
-  <si>
     <r>
-      <t xml:space="preserve">K (mg/L) -&gt; </t>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [Daten wurden manuell schon in Excel konvertiert]</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Coordinates H -&gt; </t>
     </r>
     <r>
       <rPr>
@@ -1456,241 +1747,18 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>K_mg-L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Fe (mg/L) -&gt; </t>
+      <t>Coordinates_H</t>
     </r>
     <r>
       <rPr>
-        <b/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Fe_mg-L</t>
+      <t xml:space="preserve"> [Daten wurden manuell schon in Excel konvertiert]</t>
     </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Mn (mg/L) -&gt; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Mn_mg-L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Na (mg/L) -&gt; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Na_mg-L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Mg (mg/L) -&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Mg_mg-L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Ca (mg/L) -&gt; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Ca_mg-L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Cl (mg/L) -&gt; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Cl_mg-L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">SO4 (mg/L) -&gt; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SO4_mg-l</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">HCO3 (mg/L) -&gt; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>HCO3_mg-l</t>
-    </r>
-  </si>
-  <si>
-    <t>Geothermal province -&gt; Geothermal_province</t>
-  </si>
-  <si>
-    <t>Nein, da HCO3 einwertig ist gilt meq/L = mmol/L</t>
-  </si>
-  <si>
-    <r>
-      <t>CLA flow path -&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> CLA_flow_path</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Bore/Spring -&gt; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Bore_Spring</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Mg (mg/L) -&gt; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Mg_mg-L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Ca (mg/L) -&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Ca_mg-L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>SO4 (mg/L) -&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> SO4_mg-L</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Alkalinity (meq/L) -&gt; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Alkalinity_meq-L</t>
-    </r>
-  </si>
-  <si>
-    <t>liegt in ppb vor, müsste in ppm vorliegen, Faktor / 1.000</t>
   </si>
 </sst>
 </file>
@@ -2971,7 +3039,7 @@
         <v>85</v>
       </c>
       <c r="G4" s="61" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -2991,7 +3059,7 @@
         <v>85</v>
       </c>
       <c r="G5" s="61" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
@@ -3137,7 +3205,7 @@
         <v>165</v>
       </c>
       <c r="G17" s="61" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
@@ -3157,7 +3225,7 @@
         <v>165</v>
       </c>
       <c r="G18" s="61" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
@@ -3177,7 +3245,7 @@
         <v>165</v>
       </c>
       <c r="G19" s="61" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
@@ -3197,7 +3265,7 @@
         <v>165</v>
       </c>
       <c r="G20" s="61" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
@@ -3217,7 +3285,7 @@
         <v>165</v>
       </c>
       <c r="G21" s="61" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
@@ -3234,10 +3302,10 @@
         <v>80</v>
       </c>
       <c r="F22" s="28" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="G22" s="61" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
@@ -3267,7 +3335,7 @@
         <v>165</v>
       </c>
       <c r="G24" s="61" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.25">
@@ -5184,7 +5252,7 @@
         <v>165</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
@@ -8367,7 +8435,7 @@
     <col min="5" max="5" width="29.5703125" customWidth="1"/>
     <col min="6" max="6" width="25.28515625" customWidth="1"/>
     <col min="7" max="7" width="27.140625" customWidth="1"/>
-    <col min="8" max="8" width="63.42578125" customWidth="1"/>
+    <col min="8" max="8" width="76.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -8419,7 +8487,7 @@
       <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="80" t="s">
         <v>220</v>
       </c>
       <c r="D5" t="s">
@@ -8434,7 +8502,9 @@
       <c r="G5" s="23" t="s">
         <v>222</v>
       </c>
-      <c r="H5" s="23"/>
+      <c r="H5" s="61" t="s">
+        <v>406</v>
+      </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
@@ -8456,7 +8526,7 @@
         <v>234</v>
       </c>
       <c r="H6" s="61" t="s">
-        <v>389</v>
+        <v>409</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
@@ -8479,14 +8549,14 @@
         <v>234</v>
       </c>
       <c r="H7" s="61" t="s">
-        <v>388</v>
+        <v>410</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="80" t="s">
         <v>227</v>
       </c>
       <c r="D8" t="s">
@@ -8501,13 +8571,15 @@
       <c r="G8" s="23" t="s">
         <v>222</v>
       </c>
-      <c r="H8" s="23"/>
+      <c r="H8" s="61" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="80" t="s">
         <v>228</v>
       </c>
       <c r="D9" t="s">
@@ -8522,7 +8594,9 @@
       <c r="G9" s="23" t="s">
         <v>229</v>
       </c>
-      <c r="H9" s="23"/>
+      <c r="H9" s="61" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
@@ -9024,7 +9098,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="5" scale="68" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="5" scale="65" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9535,7 +9609,7 @@
         <v>85</v>
       </c>
       <c r="G4" s="61" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -9707,7 +9781,7 @@
         <v>165</v>
       </c>
       <c r="G17" s="61" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
@@ -9727,7 +9801,7 @@
         <v>165</v>
       </c>
       <c r="G18" s="61" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
@@ -9747,7 +9821,7 @@
         <v>165</v>
       </c>
       <c r="G19" s="61" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
@@ -9767,7 +9841,7 @@
         <v>165</v>
       </c>
       <c r="G20" s="61" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
@@ -9787,7 +9861,7 @@
         <v>165</v>
       </c>
       <c r="G21" s="61" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
@@ -9807,7 +9881,7 @@
         <v>165</v>
       </c>
       <c r="G22" s="61" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
@@ -9837,7 +9911,7 @@
         <v>165</v>
       </c>
       <c r="G24" s="61" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.25">
@@ -9877,7 +9951,7 @@
         <v>165</v>
       </c>
       <c r="G27" s="61" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.25">
@@ -9897,7 +9971,7 @@
         <v>165</v>
       </c>
       <c r="G28" s="61" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.25">

</xml_diff>